<commit_message>
Add SQL Practice files
</commit_message>
<xml_diff>
--- a/excel-project/class_survey_results-1.xlsx
+++ b/excel-project/class_survey_results-1.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\data-analytics-projects-main\excel-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D25E40-C698-4419-A18C-A4E7E22C4DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B42958CE-A309-45EE-BE09-F700DD3F49DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{AD976FC9-9605-427E-8A94-DC4CC3EC4C37}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{AD976FC9-9605-427E-8A94-DC4CC3EC4C37}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
     <sheet name="class_survey_results-1" sheetId="1" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="37">
   <si>
     <t>Student ID</t>
   </si>
@@ -1445,6 +1446,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="693572976"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -1503,6 +1505,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="693572496"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
@@ -1558,6 +1561,538 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="708335184"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-NG"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-NG"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-NG"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$A$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet3!$A$2:$A$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FF09-4B1E-BA03-DA81AF31A677}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet3!$B$2:$B$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-FF09-4B1E-BA03-DA81AF31A677}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="46803407"/>
+        <c:axId val="46802447"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>65</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet3!$C$2:$C$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>77</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>82</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-FF09-4B1E-BA03-DA81AF31A677}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="46807247"/>
+        <c:axId val="46806767"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="46803407"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-NG"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="46802447"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="46802447"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-NG"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="46803407"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="46806767"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-NG"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="46807247"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="46807247"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="46806767"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -1726,6 +2261,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -2243,6 +2818,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2820,6 +3911,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87D2D30E-9BF1-FB33-6E69-3E1573C4FA34}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>166687</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F2E8E6D-7440-8291-0012-1D31D5F48E17}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3871,12 +5003,12 @@
         <v>Tablet</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N5" si="2">COUNTIF(E3:E17,M3)</f>
+        <f t="shared" ref="N3:N4" si="2">COUNTIF(E3:E17,M3)</f>
         <v>4</v>
       </c>
       <c r="O3">
-        <f>ROUND(AVERAGE(C2:C16),2)</f>
-        <v>10.07</v>
+        <f>ROUND(AVERAGE(C2:C16),1)</f>
+        <v>10.1</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -4220,8 +5352,22 @@
       <c r="F16">
         <v>86</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K16" cm="1">
+        <f t="array" ref="K16:K30">$C$2:$C$16</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K18">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B19">
         <f>CORREL($C$2:$C$16,$F$2:$F$16)</f>
         <v>0.84621555000184756</v>
@@ -4232,96 +5378,132 @@
       <c r="E19" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K19">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D20">
         <v>5</v>
       </c>
       <c r="E20">
         <v>65</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K20">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D21">
         <v>6</v>
       </c>
       <c r="E21">
         <v>70</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D22">
         <v>6</v>
       </c>
       <c r="E22">
         <v>73</v>
       </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K22">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D23">
         <v>9</v>
       </c>
       <c r="E23">
         <v>75</v>
       </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D24">
         <v>9</v>
       </c>
       <c r="E24">
         <v>77</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K24">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D25">
         <v>8</v>
       </c>
       <c r="E25">
         <v>78</v>
       </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D26">
         <v>7</v>
       </c>
       <c r="E26">
         <v>80</v>
       </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K26">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D27">
         <v>11</v>
       </c>
       <c r="E27">
         <v>82</v>
       </c>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K27">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D28">
         <v>16</v>
       </c>
       <c r="E28">
         <v>84</v>
       </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K28">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D29">
         <v>10</v>
       </c>
       <c r="E29">
         <v>85</v>
       </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K29">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D30">
         <v>10</v>
       </c>
       <c r="E30">
         <v>86</v>
       </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K30">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D31">
         <v>14</v>
       </c>
@@ -4329,7 +5511,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D32">
         <v>12</v>
       </c>
@@ -4363,6 +5545,152 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FAEC4F6-B5D1-4D15-AD22-66AB1F6C6C46}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>5</v>
+      </c>
+      <c r="C1">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>8</v>
+      </c>
+      <c r="C5">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>9</v>
+      </c>
+      <c r="C6">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="C8">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>12</v>
+      </c>
+      <c r="C11">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>13</v>
+      </c>
+      <c r="C12">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>14</v>
+      </c>
+      <c r="C13">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>15</v>
+      </c>
+      <c r="C14">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>16</v>
+      </c>
+      <c r="C15">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:C16">
+    <sortCondition ref="A1:A16"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30217A6E-C923-4466-8DE7-43500BED2FCA}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>